<commit_message>
scan: seg8 2026-10-23 20:31 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq0_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq0_2026-10-22.xlsx
@@ -1587,21 +1587,21 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>8358</v>
+        <v>8068</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>金居</t>
+          <t>全達</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>540.0856309617162</v>
+        <v>528.4336031086613</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>438.5</v>
+        <v>17.95</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1612,49 +1612,49 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>39.37036983550509</v>
+        <v>51.8269509729345</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>21.5016365977421</v>
+        <v>32.31130619351321</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>1.345283816282502</v>
+        <v>0.3125278343269877</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M22" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>-9.326652880886732</v>
+        <v>-0.04948983574958155</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>8068</v>
+        <v>8045</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>全達</t>
+          <t>達運光電</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>528.4336031086613</v>
+        <v>522.754156580491</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>17.95</v>
+        <v>54.5</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1665,13 +1665,13 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>51.8269509729345</v>
+        <v>50.90640590730123</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>32.31130619351321</v>
+        <v>17.21828636207105</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>0.3125278343269877</v>
+        <v>3.192497051227178</v>
       </c>
       <c r="K23" s="2" t="n">
         <v>1</v>
@@ -1683,31 +1683,31 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.04948983574958155</v>
+        <v>-0.1850356898191404</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>8045</v>
+        <v>8442</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>達運光電</t>
+          <t>威宏-KY</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>522.754156580491</v>
+        <v>511.4733896006021</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>54.5</v>
+        <v>48.05</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,16 +1718,16 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>50.90640590730123</v>
+        <v>57.85587132342967</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>17.21828636207105</v>
+        <v>19.51798087937892</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>3.192497051227178</v>
+        <v>0.7283386577451325</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>0</v>
@@ -1736,31 +1736,31 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-0.1850356898191404</v>
+        <v>0.08787671895771565</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>volume_break, avoid_chase, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>8442</v>
+        <v>8422</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>威宏-KY</t>
+          <t>可寧衛*</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>511.4733896006021</v>
+        <v>504.3502174668314</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>48.05</v>
+        <v>26.05</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,16 +1771,16 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>57.85587132342967</v>
+        <v>54.0504927659699</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>19.51798087937892</v>
+        <v>12.59871547862918</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.7283386577451325</v>
+        <v>1.27197822733779</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -1789,51 +1789,51 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.08787671895771565</v>
+        <v>0.1122603666706546</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>avoid_chase, liquidity_ok, foreign_buy_3d, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>8422</v>
+        <v>8908</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>可寧衛*</t>
+          <t>欣雄</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>504.3502174668314</v>
+        <v>500.8642278537419</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>26.05</v>
+        <v>40.2</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="G26" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>54.0504927659699</v>
+        <v>53.97361638023576</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>12.59871547862918</v>
+        <v>15.22478438469357</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>1.27197822733779</v>
+        <v>0.760617295114085</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -1842,51 +1842,51 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.1122603666706546</v>
+        <v>-0.005565450949512912</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, liquidity_ok, foreign_buy_3d, stronger_than_market, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, cci_momentum</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>8908</v>
+        <v>8074</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>欣雄</t>
+          <t>鉅橡</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>500.8642278537419</v>
+        <v>498.9441155752468</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>40.2</v>
+        <v>57.1</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="G27" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>53.97361638023576</v>
+        <v>53.45838566710947</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>15.22478438469357</v>
+        <v>27.10638510876368</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.760617295114085</v>
+        <v>1.620056674341036</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.005565450949512912</v>
+        <v>0.4813043395196474</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend, cci_momentum</t>
+          <t>volume_break, liquidity_ok, adx_trending, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>8074</v>
+        <v>8431</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>鉅橡</t>
+          <t>匯鑽科</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>498.9441155752468</v>
+        <v>489.8719907943196</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>57.1</v>
+        <v>62.2</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>53.45838566710947</v>
+        <v>47.60324785579318</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>27.10638510876368</v>
+        <v>29.26039297542794</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>1.620056674341036</v>
+        <v>0.8433100139456761</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.4813043395196474</v>
+        <v>-0.4819141837382799</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>volume_break, liquidity_ok, adx_trending, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>8431</v>
+        <v>8249</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>匯鑽科</t>
+          <t>菱光</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>489.8719907943196</v>
+        <v>488.89791048901</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>62.2</v>
+        <v>39.9</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,16 +1983,16 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>47.60324785579318</v>
+        <v>50.501784022382</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>29.26039297542794</v>
+        <v>12.71692574520556</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.8433100139456761</v>
+        <v>1.074079888439611</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-0.4819141837382799</v>
+        <v>0.0592468698426855</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>avoid_chase, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>8249</v>
+        <v>8358</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>菱光</t>
+          <t>金居</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>488.89791048901</v>
+        <v>480.0856309617163</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>39.9</v>
+        <v>438.5</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,29 +2036,29 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>50.501784022382</v>
+        <v>39.3703697280673</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>12.71692574520556</v>
+        <v>21.50163660845583</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>1.074079888439611</v>
+        <v>1.345283816282502</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M30" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.0592468698426855</v>
+        <v>-9.326652877521884</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scan: seg8 2026-10-26 15:54 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq0_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq0_2026-10-22.xlsx
@@ -444,7 +444,7 @@
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>61.50171368016709</v>
+        <v>61.50171373182884</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>30.53874863557703</v>
+        <v>30.53874866596949</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1.797238866899151</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>1.273688031207344</v>
+        <v>1.273688030039263</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>63.4394239481556</v>
+        <v>63.4394241817897</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>11.54868701233453</v>
+        <v>11.5486871381744</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.932041140472446</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.2032258086768626</v>
+        <v>0.2032258084172884</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>68.32600295464555</v>
+        <v>68.32600301713751</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>51.89439413687717</v>
+        <v>51.89439419265171</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.649331275218209</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.4737129370476854</v>
+        <v>0.4737129367881139</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>57.77468787032137</v>
+        <v>57.77468794023336</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>23.90673817269061</v>
+        <v>23.90673824562103</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>2.461429822034452</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-0.512646979270675</v>
+        <v>-0.5126469797898273</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>84.28342206643244</v>
+        <v>84.28342209042978</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>48.4530097721499</v>
+        <v>48.45301000807365</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>5.267636097406806</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.7206381115226961</v>
+        <v>0.7206381112761004</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>723.5012411319307</v>
+        <v>723.5012411319306</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1560</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>52.23455205649191</v>
+        <v>52.23455206766463</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>38.64801622623421</v>
+        <v>38.64801629521836</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.389343383413787</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-20.31701356580082</v>
+        <v>-20.31701357099193</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>694.1130176441686</v>
+        <v>694.1130176441685</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>265</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>56.81367649244098</v>
+        <v>56.81367658368842</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>16.99152253386061</v>
+        <v>16.99152257505579</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.045550351898062</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.4546121121406896</v>
+        <v>0.454612111102402</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>686.937088055392</v>
+        <v>686.9370880553919</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>83.8</v>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>45.99428690380058</v>
+        <v>45.99428695321446</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>12.69141974046996</v>
+        <v>12.69141991148065</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.6919213594621682</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.1935761707560657</v>
+        <v>0.1935761704964882</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>53.47443679941819</v>
+        <v>53.4744366656749</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>24.50155145324227</v>
+        <v>24.50155138019889</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0.8282646549768207</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1.645833328514684</v>
+        <v>1.64583332721682</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>55.12933768297461</v>
+        <v>55.12933773716534</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>31.95323294619063</v>
+        <v>31.95323302397382</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.375083957017453</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-0.05649180259318531</v>
+        <v>-0.05649180267105935</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>72.51099781675981</v>
+        <v>72.51099769319148</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>37.00919184516221</v>
+        <v>37.00919195497092</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.8289482352553651</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.2568998042638775</v>
+        <v>-0.2568998043528503</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>45.5395746087177</v>
+        <v>45.53957463082892</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>21.17566591491102</v>
+        <v>21.17566613302319</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.7298391083725189</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-23.46145382668089</v>
+        <v>-23.46145383161297</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>61.36656790714808</v>
+        <v>61.3665677828796</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>40.58533084160902</v>
+        <v>40.58533095372463</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.202411050093229</v>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>51.43641490149892</v>
+        <v>51.43641500382593</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>18.18612494402323</v>
+        <v>18.18612503349156</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>1.308516129253</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.1438850158700735</v>
+        <v>0.1438850155715661</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>614.372367837201</v>
+        <v>614.3723678372006</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>13.15</v>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>52.22730823298386</v>
+        <v>52.22730822503998</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>23.46738399753534</v>
+        <v>23.46738390560164</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>10.19299099907937</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.2041250717883042</v>
+        <v>0.2041250718272411</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>39.98360427191673</v>
+        <v>39.98360427322074</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>28.94346984800228</v>
+        <v>28.94346993347793</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.3595557409180549</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>-3.454916944318438</v>
+        <v>-3.454916944409292</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>54.15670710931615</v>
+        <v>54.15670729667846</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>15.4075481230038</v>
+        <v>15.40754798236666</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.9748786120322123</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1.430281991943209</v>
+        <v>1.430281990775133</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>51.50418820446403</v>
+        <v>51.50418819056291</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>20.20208429788623</v>
+        <v>20.20208431641569</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>5.853529023135771</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.09256653412948324</v>
+        <v>0.09256653411650462</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>53.67514934115864</v>
+        <v>53.67514933433792</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>41.58302253948924</v>
+        <v>41.58302266699273</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>1.91652321707221</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.3665664797871413</v>
+        <v>0.366566479670305</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>49.24034778975236</v>
+        <v>49.24034782780798</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>30.8530375327063</v>
+        <v>30.8530374509283</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.37520077790923</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-0.2342485491350657</v>
+        <v>-0.2342485493946358</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>528.4336031086613</v>
+        <v>528.4336031086614</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>17.95</v>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>51.8269509729345</v>
+        <v>51.82695093379393</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>32.31130619351321</v>
+        <v>32.31130618802195</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.3125278343269877</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>-0.04948983574958155</v>
+        <v>-0.04948983584043432</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>522.754156580491</v>
+        <v>522.7541565804908</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>54.5</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>50.90640590730123</v>
+        <v>50.90640579040686</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>17.21828636207105</v>
+        <v>17.21828633704896</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>3.192497051227178</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.1850356898191404</v>
+        <v>-0.1850356913765788</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>57.85587132342967</v>
+        <v>57.85587131126581</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>19.51798087937892</v>
+        <v>19.51798095088931</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.7283386577451325</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.08787671895771565</v>
+        <v>0.08787671919133233</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>54.0504927659699</v>
+        <v>54.05049187495794</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>12.59871547862918</v>
+        <v>12.59871554434059</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>1.27197822733779</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.1122603666706546</v>
+        <v>0.1122603671155191</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>500.8642278537419</v>
+        <v>500.8642278537417</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>40.2</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>53.97361638023576</v>
+        <v>53.97361633735492</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>15.22478438469357</v>
+        <v>15.22478447187373</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.760617295114085</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>-0.005565450949512912</v>
+        <v>-0.005565450914197662</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>53.45838566710947</v>
+        <v>53.45838567121151</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>27.10638510876368</v>
+        <v>27.10638527073353</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.620056674341036</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.4813043395196474</v>
+        <v>0.4813043390264591</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>47.60324785579318</v>
+        <v>47.603247879543</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>29.26039297542794</v>
+        <v>29.26039307133874</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.8433100139456761</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-0.4819141837382799</v>
+        <v>-0.4819141839848768</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>488.89791048901</v>
+        <v>488.8979104889937</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>39.9</v>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>50.501784022382</v>
+        <v>50.50178363646307</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>12.71692574520556</v>
+        <v>12.71692597047239</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>1.074079888439611</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.0592468698426855</v>
+        <v>0.05924687023204278</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>39.3703697280673</v>
+        <v>39.37036986652829</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>21.50163660845583</v>
+        <v>21.50163664777957</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>1.345283816282502</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-9.326652877521884</v>
+        <v>-9.32665288310271</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>42.11470591032023</v>
+        <v>42.11470551030486</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>14.11400879971829</v>
+        <v>14.11400893755898</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.3423318568761622</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.04750364181697075</v>
+        <v>0.04750364199866763</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>475.332077296038</v>
+        <v>475.3320772960382</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>61.8</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>44.35447907205993</v>
+        <v>44.35447911731011</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>13.0082082316765</v>
+        <v>13.00820832998108</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.7345672408259335</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.1066589073529786</v>
+        <v>0.1066589062108509</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2181,7 +2181,7 @@
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>474.8731161740699</v>
+        <v>474.8731161740701</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>24.35</v>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>47.11976746900975</v>
+        <v>47.1197676563804</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>26.81735301615809</v>
+        <v>26.81735316039164</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.7158299275388671</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.07436470207526158</v>
+        <v>0.07436470178972998</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>57.65549508287145</v>
+        <v>57.655495290173</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>15.58556541371103</v>
+        <v>15.58556537373398</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.9334858343414639</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.03441299823535342</v>
+        <v>0.03441299821458883</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>52.26987112182793</v>
+        <v>52.26987111771572</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>29.94338313883316</v>
+        <v>29.94338307506749</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.3688200112431441</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-0.01366763527767259</v>
+        <v>-0.01366763528286369</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>40.06283616037017</v>
+        <v>40.06283616390967</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>16.71172425404793</v>
+        <v>16.71172429484598</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.6229934965662307</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-19.20419345325934</v>
+        <v>-19.20419345481692</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>442.4270914848674</v>
+        <v>442.4270914848673</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>105</v>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>41.8448105103401</v>
+        <v>41.8448105376739</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>24.88002212530082</v>
+        <v>24.88002216419947</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.8087478741629615</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-1.871138257232515</v>
+        <v>-1.871138257277019</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,7 +2460,7 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>46.11781227019094</v>
+        <v>46.11781235547103</v>
       </c>
       <c r="I38" s="2" t="n">
         <v>15.806142562236</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-0.052219510574884</v>
+        <v>-0.05221951066573907</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>47.2361013599111</v>
+        <v>47.23610138580127</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>28.78978295651203</v>
+        <v>28.78978311085551</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.1746813324909014</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-1.552702538287534</v>
+        <v>-1.552702538676902</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>45.24331609992868</v>
+        <v>45.24331630944906</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>18.08951202431034</v>
+        <v>18.08951226580136</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>1.04372566316102</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-0.8614604622876034</v>
+        <v>-0.8614604637152564</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>42.04131892583695</v>
+        <v>42.04131901071852</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>26.72678010528671</v>
+        <v>26.72678014602368</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.335975109515038</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.008366818617654426</v>
+        <v>-0.008366818773398399</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>54.69770652415691</v>
+        <v>54.69770648794883</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>15.43045642312898</v>
+        <v>15.43045636843283</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>1.023829733570677</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.02129136445455948</v>
+        <v>0.02129136438783163</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>44.01760702597932</v>
+        <v>44.01760703854805</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>21.33494807302529</v>
+        <v>21.33494798698741</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>1.031595582424542</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-2.410040753142936</v>
+        <v>-2.410040754155257</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>18.14864276482068</v>
+        <v>18.14864275051552</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>64.47578397068102</v>
+        <v>64.47578399552995</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.3745321416476234</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.2834025114152681</v>
+        <v>0.2834025114022882</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>50.14212315923367</v>
+        <v>50.14212327714911</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>27.207107838658</v>
+        <v>27.20710785675488</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.8661811693613135</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.05163714083488474</v>
+        <v>-0.05163714102956696</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>46.24856669141653</v>
+        <v>46.24856619186897</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>30.0945952420744</v>
+        <v>30.09459504828553</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.5985639926676436</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-0.008811208164298734</v>
+        <v>-0.008811208073448538</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>38.2742510360826</v>
+        <v>38.27425107882759</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>27.17132178648096</v>
+        <v>27.1713216926055</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>1.248760791605791</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.06347425185174771</v>
+        <v>0.06347425177387189</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>44.16815941628943</v>
+        <v>44.1681594067116</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>30.88617359621557</v>
+        <v>30.88617360007971</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.2927270027077626</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.9076564463788017</v>
+        <v>-0.9076564463268855</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>43.10934081404089</v>
+        <v>43.10934075832134</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>28.86344144011566</v>
+        <v>28.86344158095253</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.4570071315006982</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.08714042171964814</v>
+        <v>0.08714042178454223</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>43.94967714175216</v>
+        <v>43.94967721138834</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>11.16674471712932</v>
+        <v>11.16674482071125</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.7724666649442282</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.01224073236541031</v>
+        <v>-0.01224073240434776</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,7 +3149,7 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>47.77985932318072</v>
+        <v>47.77985935728047</v>
       </c>
       <c r="I51" s="2" t="n">
         <v>13.84089946326911</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.4064827947650409</v>
+        <v>-0.4064827929479835</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>369.649701269184</v>
+        <v>369.6497012691836</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>44.4</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>50.18577418593332</v>
+        <v>50.18577418024257</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>7.474352852799967</v>
+        <v>7.474352903642559</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.6480589829337459</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.003918341179372398</v>
+        <v>-0.003918341158777761</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>45.80555369973113</v>
+        <v>45.80555365200031</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>24.32964765407042</v>
+        <v>24.3296476542161</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.5301168375327538</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-1.470456768614619</v>
+        <v>-1.470456768744411</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>355.8634049635208</v>
+        <v>355.863404963521</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>28.2</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>44.90268733273678</v>
+        <v>44.90268730373873</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>19.14537767042352</v>
+        <v>19.14537746212603</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>1.870816255095116</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.06862061706016942</v>
+        <v>0.06862061532379116</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>349.4688240525207</v>
+        <v>349.4688240525206</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>81.3</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>33.63506175925728</v>
+        <v>33.6350617425975</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>31.47339944374181</v>
+        <v>31.4733995995488</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.7577526632333104</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.2866701129458038</v>
+        <v>0.2866701126083626</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>44.02262254480209</v>
+        <v>44.02262255554795</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>16.37298262256741</v>
+        <v>16.37298281884591</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>1.551163132568259</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-2.461029626340804</v>
+        <v>-2.46102962674316</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>38.50390317791035</v>
+        <v>38.50390316732724</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>13.67564520334494</v>
+        <v>13.67564526262068</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.7801535217607619</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.1381623608358448</v>
+        <v>-0.1381623606411645</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>344.5105095668256</v>
+        <v>344.5105095668258</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>67.7</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>46.32850574735829</v>
+        <v>46.3285059041681</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>23.32840468162406</v>
+        <v>23.32840468587395</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.2193044977159437</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.1042137859648411</v>
+        <v>0.1042137844074038</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>338.4180120933565</v>
+        <v>338.4180120933575</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>177</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>26.54916420526433</v>
+        <v>26.54916422087081</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>26.48924166519385</v>
+        <v>26.48924177055491</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.750165316765388</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-1.352097255275394</v>
+        <v>-1.352097255742629</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>41.32348396896128</v>
+        <v>41.32348398716119</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>19.18635301617674</v>
+        <v>19.18635307887863</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.4009966140390467</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.566202864935148</v>
+        <v>-0.5662028650649406</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>330.8222654617339</v>
+        <v>330.8222654617473</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>19.45</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>47.46911833715647</v>
+        <v>47.46911794695054</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>13.28982039802381</v>
+        <v>13.28982047966328</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.7996286015494279</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.02403068634437638</v>
+        <v>-0.02403068622756863</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>46.82090167592073</v>
+        <v>46.82090170459927</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>18.41214571832975</v>
+        <v>18.41214582093743</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.2286572105170016</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.5644588581065276</v>
+        <v>-0.5644588582103581</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3771,7 +3771,7 @@
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>325.2703774014066</v>
+        <v>325.2703774014073</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>74.3</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>36.6021827801613</v>
+        <v>36.60218295098283</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>17.65194091910938</v>
+        <v>17.65194106342507</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.3678364364167878</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.8149528926226455</v>
+        <v>-0.814952893531141</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>45.93876060191161</v>
+        <v>45.93876062673137</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>30.42464127945239</v>
+        <v>30.42464118011972</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.9079523187005889</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-12.29579160873512</v>
+        <v>-12.29579161094156</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>39.28043422801703</v>
+        <v>39.28043427404442</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>21.25291068131371</v>
+        <v>21.25291059009146</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.2102217793858742</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-1.7244927164489</v>
+        <v>-1.724492716345079</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>50.1375894311203</v>
+        <v>50.13758956766841</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>24.78789281735936</v>
+        <v>24.78789276130733</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.5386565802160797</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.2147468412571246</v>
+        <v>-0.214746841168152</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>51.63431286601788</v>
+        <v>51.63431288306025</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>32.20069294572093</v>
+        <v>32.20069310143391</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4025606890735801</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.1738023745228495</v>
+        <v>0.1738023744839139</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,7 +4050,7 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>42.0553924887703</v>
+        <v>42.05539251160287</v>
       </c>
       <c r="I68" s="2" t="n">
         <v>17.07120798668088</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.2234359646924797</v>
+        <v>-0.2234359651077971</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>309.4934264266204</v>
+        <v>309.4934264266202</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>13.6</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>37.02351431364069</v>
+        <v>37.02351429036546</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>39.95172834068127</v>
+        <v>39.95172840417597</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.3736175337522871</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.02266553523138232</v>
+        <v>0.02266553524436077</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>49.27933152608298</v>
+        <v>49.27933149612411</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>26.54081338911667</v>
+        <v>26.54081336346389</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.3021083385677799</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.01279963998204655</v>
+        <v>0.01279963991715352</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>37.7371002647916</v>
+        <v>37.73710052447799</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>7.578239876228462</v>
+        <v>7.578239942429825</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.6903404347948481</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.03234129096762617</v>
+        <v>0.03234129013699305</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>302.2398939512981</v>
+        <v>302.2398939513393</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>41.3</v>
@@ -4265,7 +4265,7 @@
         <v>39.50043926202966</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>12.36700616281097</v>
+        <v>12.36700622319114</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.7583543671928425</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.1377093084242831</v>
+        <v>-0.1377093085410869</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4301,7 +4301,7 @@
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>302.0798237348228</v>
+        <v>302.0798237348229</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>19.75</v>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>40.00589240939506</v>
+        <v>40.00589299954748</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>20.07196158517669</v>
+        <v>20.0719619942676</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.8314611749119293</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.04729823627193598</v>
+        <v>-0.04729823666129725</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>48.02539057384062</v>
+        <v>48.02539058810623</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>31.6094303923092</v>
+        <v>31.60943063434203</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.6095204455587635</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.003609390469838519</v>
+        <v>-0.003609390500986409</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>297.846306055576</v>
+        <v>297.8463060555758</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>764</v>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>26.8680443932701</v>
+        <v>26.86804444221994</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>26.31862794579234</v>
+        <v>26.31862807322475</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>1.065416436243068</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-4.333035119065524</v>
+        <v>-4.333035127112247</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>296.9000702312881</v>
+        <v>296.9000702312807</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>19.5</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>40.93627461929126</v>
+        <v>40.93627450698609</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>23.72262424359502</v>
+        <v>23.72262429826972</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.8683105312073887</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.1198481075571711</v>
+        <v>-0.1198481074273851</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>24.76832143070415</v>
+        <v>24.76832138047335</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>50.17979981143835</v>
+        <v>50.17979962236757</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.1761600127597839</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.03344874298914979</v>
+        <v>-0.03344874297617167</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>289.3931012764519</v>
+        <v>289.3931012764559</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>20.15</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>35.41486826693</v>
+        <v>35.41486829247042</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>16.9990781010153</v>
+        <v>16.99907819781869</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.8229910077504513</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.07603336313274256</v>
+        <v>-0.0760333632884852</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>50.49351130759196</v>
+        <v>50.49351134911474</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>5.738456898058106</v>
+        <v>5.73845682913478</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>1.238615172562904</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-1.945536003605831</v>
+        <v>-1.945536004825834</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>276.7946915117269</v>
+        <v>276.7946915117267</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>46.7</v>
@@ -4686,7 +4686,7 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>42.8538040646361</v>
+        <v>42.85380403458104</v>
       </c>
       <c r="I80" s="2" t="n">
         <v>10.10055283827799</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.3346762826427275</v>
+        <v>-0.3346762827984709</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4725,7 +4725,7 @@
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>271.5280819589136</v>
+        <v>271.5280819589134</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>26.2</v>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>28.12497145506624</v>
+        <v>28.12497177823154</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>43.98126040941865</v>
+        <v>43.98126014125751</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.1260589222536288</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.05023570431339019</v>
+        <v>0.05023570405381628</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>35.81367277437735</v>
+        <v>35.81367276691375</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>26.97669110080937</v>
+        <v>26.97669105808152</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.4312436186957446</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-1.479100798155162</v>
+        <v>-1.479100798129205</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>33.91437619995682</v>
+        <v>33.91437623029201</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>20.53228601583493</v>
+        <v>20.53228615543403</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.4057153361421413</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-3.347800659678913</v>
+        <v>-3.347800660431654</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>264.0016706486825</v>
+        <v>264.001670648683</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>20.35</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>33.98528292733529</v>
+        <v>33.98528326136606</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>35.96020164992936</v>
+        <v>35.96020156185598</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>1.244751897517626</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.03543465292494752</v>
+        <v>-0.03543465313260941</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>51.65384851728513</v>
+        <v>51.65384851343826</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>21.25793878156007</v>
+        <v>21.25793869606789</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.1145242560780299</v>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>258.1205648875547</v>
+        <v>258.1205648875545</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>32.55</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>43.83377369144866</v>
+        <v>43.83377461967024</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>24.17382216191816</v>
+        <v>24.17382213224707</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.4968641409156804</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.3165838950817156</v>
+        <v>-0.3165838958085204</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>256.2166676300438</v>
+        <v>256.2166676300444</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>98.5</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>54.80028013304411</v>
+        <v>54.800279927151</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>18.28257213565397</v>
+        <v>18.28257218757575</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.963719827376367</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.7843235392912042</v>
+        <v>0.7843235394209975</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>50.38294863544596</v>
+        <v>50.38294863352041</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>4.623676407384895</v>
+        <v>4.623676406529136</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.5815954787037995</v>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>253.560207681737</v>
+        <v>253.5602076817368</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>125</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>39.31770866750764</v>
+        <v>39.31770868245531</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>23.06136422662244</v>
+        <v>23.06136436378518</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.3738271444984303</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-2.181594198912425</v>
+        <v>-2.181594199691157</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>244.746306237526</v>
+        <v>244.7463062375292</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>44.5</v>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>42.36321757150434</v>
+        <v>42.36321756909849</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>18.75067650162195</v>
+        <v>18.75067654923309</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.3253733246469661</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.5757832509683487</v>
+        <v>-0.5757832509943052</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>41.31554962470234</v>
+        <v>41.31554964942543</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>12.84795210036102</v>
+        <v>12.84795213917887</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.4923774439834016</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.3053859219726627</v>
+        <v>-0.3053859219986216</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>37.84693186772684</v>
+        <v>37.84693190428838</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>15.65089644938006</v>
+        <v>15.65089672684538</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.748161642941366</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-2.677513720652759</v>
+        <v>-2.677513722988849</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5350,21 +5350,21 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>8466</v>
+        <v>8488</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>美吉吉-KY</t>
+          <t>吉源-KY</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>238.593012589109</v>
+        <v>239.0701513992827</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>14.9</v>
+        <v>9.24</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>45.43712547378522</v>
+        <v>49.52163055940701</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>15.98701960763826</v>
+        <v>22.51632876046137</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.5657884665941212</v>
+        <v>1.281590585841818</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.01510060473494661</v>
+        <v>0.1055033996341257</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>8087</v>
+        <v>8466</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>華鎂鑫</t>
+          <t>美吉吉-KY</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>237.5603722103006</v>
+        <v>238.593012589109</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>22.4</v>
+        <v>14.9</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>47.03531354258766</v>
+        <v>45.4371256562962</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>3.870230716153533</v>
+        <v>15.98701958534786</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.06548518569400559</v>
+        <v>0.5657884665941212</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.04944592067754183</v>
+        <v>-0.01510060476090434</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>9136</v>
+        <v>8087</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>巨騰-DR</t>
+          <t>華鎂鑫</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>237.3675693885414</v>
+        <v>237.5603722103005</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>7.68</v>
+        <v>22.4</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,16 +5481,16 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>15.69743694398886</v>
+        <v>47.03531368844032</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>21.72441320492994</v>
+        <v>3.870230723404996</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>3.421454116568932</v>
+        <v>0.06548518569400559</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.06152308710295501</v>
+        <v>-0.0494459210409437</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>volume_break, avoid_chase, adx_trending</t>
+          <t>avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>8049</v>
+        <v>9136</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>晶采</t>
+          <t>巨騰-DR</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>233.0357548661147</v>
+        <v>237.3675693885414</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>23.9</v>
+        <v>7.68</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>33.36078598737454</v>
+        <v>15.69743698809964</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>16.52441067878046</v>
+        <v>21.72441319197193</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>1.109337734460097</v>
+        <v>3.421454116568932</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.04219644773433781</v>
+        <v>-0.06152308711852905</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, stronger_than_market</t>
+          <t>volume_break, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>8374</v>
+        <v>8049</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>羅昇</t>
+          <t>晶采</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>227.2064023171834</v>
+        <v>233.0357548661148</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>70.5</v>
+        <v>23.9</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>32.59237314145361</v>
+        <v>33.36078602466803</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>18.33774778354003</v>
+        <v>16.52441081117911</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>1.483481291786557</v>
+        <v>1.109337734460097</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.2881682990702772</v>
+        <v>-0.04219644779923101</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5615,21 +5615,21 @@
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>8091</v>
+        <v>8374</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>翔名</t>
+          <t>羅昇</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>226.6045878300167</v>
+        <v>227.2064023171833</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>200</v>
+        <v>70.5</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>34.83051931479434</v>
+        <v>32.59237327679445</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>14.65965332830009</v>
+        <v>18.33774776030779</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>1.350645171258896</v>
+        <v>1.483481291786557</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-2.401277662143217</v>
+        <v>-0.2881683004979345</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok</t>
+          <t>avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>8131</v>
+        <v>8091</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>福懋科</t>
+          <t>翔名</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>224.2324896292062</v>
+        <v>226.60458783002</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>60.7</v>
+        <v>200</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>42.81572558350699</v>
+        <v>34.83051939179053</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>15.94898311630488</v>
+        <v>14.659653357029</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.5436698798860434</v>
+        <v>1.350645171258896</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.4495956370355274</v>
+        <v>-2.401277663960208</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>8455</v>
+        <v>8131</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>大拓-KY</t>
+          <t>福懋科</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>221.4752405649225</v>
+        <v>224.2324896291973</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>0</v>
+        <v>60.7</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>41.54577427354884</v>
+        <v>42.81572559001732</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>9.381552555927289</v>
+        <v>15.94898320783668</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0</v>
+        <v>0.5436698798860434</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.5790421243049675</v>
+        <v>-0.4495956370874426</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>obv_uptrend, mfi_strong</t>
+          <t>avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>8121</v>
+        <v>8455</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>越峰</t>
+          <t>大拓-KY</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>220.0969304012751</v>
+        <v>221.4752405649225</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>28.8</v>
+        <v>0</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>42.3381523432583</v>
+        <v>41.54577426277354</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>24.36864464017634</v>
+        <v>9.381552307582728</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.4307129207862044</v>
+        <v>0</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.4964161951325834</v>
+        <v>-0.5790421242790109</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, adx_trending, mfi_strong</t>
+          <t>obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>8043</v>
+        <v>8121</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>蜜望實</t>
+          <t>越峰</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>216.7625187200225</v>
+        <v>220.0969304012787</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>132</v>
+        <v>28.8</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>44.4247991329954</v>
+        <v>42.33815217051502</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>16.68096045311624</v>
+        <v>24.36864468633437</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.697833294412044</v>
+        <v>0.4307129207862044</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.7924920191253623</v>
+        <v>-0.4964161948730111</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok</t>
+          <t>avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>8478</v>
+        <v>8043</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>東哥遊艇</t>
+          <t>蜜望實</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>215.7705829046616</v>
+        <v>216.7625187200225</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>128.5</v>
+        <v>132</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,16 +5905,16 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>19.73839940554628</v>
+        <v>44.42479914754244</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>21.05455592012304</v>
+        <v>16.68096046317009</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>2.977058290466164</v>
+        <v>0.697833294412044</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.896610269447808</v>
+        <v>-0.7924920194498373</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>volume_break, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>8114</v>
+        <v>8478</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>振樺電</t>
+          <t>東哥遊艇</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>213.1119035547726</v>
+        <v>215.7705829046616</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>178</v>
+        <v>128.5</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,16 +5958,16 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>44.55643530374331</v>
+        <v>19.73839977360663</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>15.08285086447609</v>
+        <v>21.05455586292065</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>1.070775557214398</v>
+        <v>2.977058290466164</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.6491751605031917</v>
+        <v>-0.8966102716541926</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, stronger_than_market</t>
+          <t>volume_break, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>8481</v>
+        <v>8114</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>政伸</t>
+          <t>振樺電</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>212.6587828790158</v>
+        <v>213.1119035547726</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>40.05</v>
+        <v>178</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,16 +6011,16 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>39.52979430332983</v>
+        <v>44.55643529092183</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>16.06169498931555</v>
+        <v>15.08285084591003</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.8395852968897267</v>
+        <v>1.070775557214398</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L105" s="2" t="n">
         <v>0</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.05714974777986176</v>
+        <v>0.6491751576478841</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6039,21 +6039,21 @@
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>8291</v>
+        <v>8481</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>尚茂</t>
+          <t>政伸</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>201.8857501771712</v>
+        <v>212.6587828790156</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>23.2</v>
+        <v>40.05</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>38.68801316322939</v>
+        <v>39.52979441482393</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>18.79162327717224</v>
+        <v>16.0616949236978</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.3369283660276646</v>
+        <v>0.8395852968897267</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.3482249730297058</v>
+        <v>-0.05714974789666832</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6092,21 +6092,21 @@
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>8176</v>
+        <v>8291</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>智捷</t>
+          <t>尚茂</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>196.9963980211895</v>
+        <v>201.8857501771712</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>9.699999999999999</v>
+        <v>23.2</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>45.36114114759349</v>
+        <v>38.68801316322939</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>17.69447041164113</v>
+        <v>18.79162327717224</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.2062662338911171</v>
+        <v>0.3369283660276646</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.0112603899759063</v>
+        <v>-0.3482249730297058</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6145,21 +6145,21 @@
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>9955</v>
+        <v>8176</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>佳龍</t>
+          <t>智捷</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>184.4653787851462</v>
+        <v>196.9963980211895</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>21.75</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,16 +6170,16 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>30.08629124922865</v>
+        <v>45.36114131898143</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>16.25319487239776</v>
+        <v>17.69447047091241</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>4.34653787851462</v>
+        <v>0.2062662338911171</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.1439504956958363</v>
+        <v>0.01126038992399189</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>volume_break, avoid_chase</t>
+          <t>avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>8488</v>
+        <v>9955</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>吉源-KY</t>
+          <t>佳龍</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>179.0701513992827</v>
+        <v>184.4653787851462</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>9.24</v>
+        <v>21.75</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,16 +6223,16 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>49.52162881174859</v>
+        <v>30.08629146061122</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>22.51632413287075</v>
+        <v>16.2531948047989</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>1.281590585841818</v>
+        <v>4.34653787851462</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L109" s="2" t="n">
         <v>0</v>
@@ -6241,11 +6241,11 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.1055034025932659</v>
+        <v>-0.1439504955530714</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, adx_trending</t>
+          <t>volume_break, avoid_chase</t>
         </is>
       </c>
     </row>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>39.35144224666637</v>
+        <v>39.35144233586585</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>12.43360487538565</v>
+        <v>12.43360502172857</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.8463595253290574</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.06077418338961244</v>
+        <v>-0.06077418353378095</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>40.81778822276759</v>
+        <v>40.81778808623167</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>18.26757285186446</v>
+        <v>18.26757285832872</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.8095017441737926</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.1120079416010807</v>
+        <v>-0.1120079416400159</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>159.3744542584213</v>
+        <v>159.3744542584215</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>25.7</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>34.34670875010561</v>
+        <v>34.34670886196825</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>24.01437835449163</v>
+        <v>24.01437842929512</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.7812393633364673</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.1677220522503112</v>
+        <v>-0.1677220524579703</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>34.38874507774622</v>
+        <v>34.3887451989589</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>20.25953163164248</v>
+        <v>20.25953174821339</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>1.432971404249287</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.1165597917380517</v>
+        <v>-0.1165597919716665</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>45.72098934670063</v>
+        <v>45.72098936937811</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>10.98233253318759</v>
+        <v>10.98233258518944</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.6110869998767769</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.08801990034295065</v>
+        <v>-0.08801990038189146</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>153.2380025856973</v>
+        <v>153.2380025856971</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>225.5</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>42.63571428253263</v>
+        <v>42.63571438201638</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>6.805051756514268</v>
+        <v>6.805051810590511</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>1.532711222355678</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-2.38542786088022</v>
+        <v>-2.385427868927003</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>43.46139661999138</v>
+        <v>43.46139615292083</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>13.32812682536344</v>
+        <v>13.32812679622607</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.7739671052068966</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.03284155274729383</v>
+        <v>-0.03284155341458872</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>118.0659889900678</v>
+        <v>118.0659889900677</v>
       </c>
       <c r="E117" s="2" t="n">
         <v>87.5</v>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>35.50775784257881</v>
+        <v>35.50775766789729</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>16.90053595938348</v>
+        <v>16.90053599948205</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>1.101770488523073</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.08898545820215942</v>
+        <v>-0.08898545778684763</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>23.66743978528874</v>
+        <v>23.66743973869228</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>16.33251113327424</v>
+        <v>16.3325111402477</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>1.017304367681117</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.2790486966083741</v>
+        <v>-0.2790486965564465</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>104.7094380878896</v>
+        <v>104.7094380878897</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>12.1</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>37.08367383992994</v>
+        <v>37.08367391625161</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>11.53810269786869</v>
+        <v>11.53810276170083</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.6720828767220302</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.01753516379144993</v>
+        <v>-0.01753516390825852</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>104.3631957117796</v>
+        <v>104.3631957117807</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>37.6</v>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>33.84733026715226</v>
+        <v>33.84733019979352</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>19.31726153212624</v>
+        <v>19.31726155362415</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>1.663421211349669</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.02069686112028934</v>
+        <v>-0.02069686114624836</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg8 2026-10-27 00:08 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq0_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq0_2026-10-22.xlsx
@@ -444,7 +444,7 @@
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>61.50171373182884</v>
+        <v>61.50171396138025</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>30.53874866596949</v>
+        <v>30.53874868802219</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1.797238866899151</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>1.273688030039263</v>
+        <v>1.273688029058057</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>63.4394241817897</v>
+        <v>63.43942429906703</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>11.5486871381744</v>
+        <v>11.54868715398477</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.932041140472446</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.2032258084172884</v>
+        <v>0.2032258083612198</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>68.32600301713751</v>
+        <v>68.32600306057498</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>51.89439419265171</v>
+        <v>51.89439442631608</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.649331275218209</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.4737129367881139</v>
+        <v>0.4737129366899944</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>57.77468794023336</v>
+        <v>57.77468810987462</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>23.90673824562103</v>
+        <v>23.90673828225631</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>2.461429822034452</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>-0.5126469797898273</v>
+        <v>-0.5126469799860577</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>84.28342209042978</v>
+        <v>84.28342229412129</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>48.45301000807365</v>
+        <v>48.45301008202495</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>5.267636097406806</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.7206381112761004</v>
+        <v>0.7206381110518265</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>723.5012411319306</v>
+        <v>723.5012411319302</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>1560</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>52.23455206766463</v>
+        <v>52.2345520508196</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>38.64801629521836</v>
+        <v>38.64801635190123</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.389343383413787</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>-20.31701357099193</v>
+        <v>-20.31701357379536</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>694.1130176441685</v>
+        <v>694.1130176441686</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>265</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>56.81367658368842</v>
+        <v>56.81367662973916</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>16.99152257505579</v>
+        <v>16.99152254789433</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.045550351898062</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.454612111102402</v>
+        <v>0.454612110962211</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>686.9370880553919</v>
+        <v>686.937088055392</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>83.8</v>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>45.99428695321446</v>
+        <v>45.99428700279974</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>12.69141991148065</v>
+        <v>12.69142002049809</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.6919213594621682</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.1935761704964882</v>
+        <v>0.1935761704123905</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>53.4744366656749</v>
+        <v>53.47443693933425</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>24.50155138019889</v>
+        <v>24.50155121242718</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0.8282646549768207</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>1.64583332721682</v>
+        <v>1.645833324413421</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>55.12933773716534</v>
+        <v>55.12933768571927</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>31.95323302397382</v>
+        <v>31.95323305581445</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.375083957017453</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-0.05649180267105935</v>
+        <v>-0.05649180262900466</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1068,7 +1068,7 @@
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>665.0905895082298</v>
+        <v>665.0905895082299</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>15.4</v>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>72.51099769319148</v>
+        <v>72.51099808545953</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>37.00919195497092</v>
+        <v>37.00919207063972</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.8289482352553651</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.2568998043528503</v>
+        <v>-0.2568998045450317</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>45.53957463082892</v>
+        <v>45.53957462686024</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>21.17566613302319</v>
+        <v>21.17566634145527</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.7298391083725189</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>-23.46145383161297</v>
+        <v>-23.46145383273422</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>61.3665677828796</v>
+        <v>61.36656801780887</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>40.58533095372463</v>
+        <v>40.58533105398158</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.202411050093229</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>-0.07237484734780675</v>
+        <v>-0.07237484762814683</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>51.43641500382593</v>
+        <v>51.43641498946243</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>18.18612503349156</v>
+        <v>18.18612504700523</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>1.308516129253</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.1438850155715661</v>
+        <v>0.1438850157678101</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>614.3723678372006</v>
+        <v>614.3723678372007</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>13.15</v>
@@ -1297,7 +1297,7 @@
         <v>52.22730822503998</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>23.46738390560164</v>
+        <v>23.46738402534073</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>10.19299099907937</v>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>39.98360427322074</v>
+        <v>39.98360432626828</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>28.94346993347793</v>
+        <v>28.94347001778629</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.3595557409180549</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>-3.454916944409292</v>
+        <v>-3.454916944479373</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>585.7223040473233</v>
+        <v>585.7223040473232</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>250</v>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>54.15670729667846</v>
+        <v>54.15670717577564</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>15.40754798236666</v>
+        <v>15.40754794193491</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.9748786120322123</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>1.430281990775133</v>
+        <v>1.430281992176828</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>51.50418819056291</v>
+        <v>51.50418768156867</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>20.20208431641569</v>
+        <v>20.20208431072036</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>5.853529023135771</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.09256653411650462</v>
+        <v>0.09256653400437043</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>53.67514933433792</v>
+        <v>53.67514935213277</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>41.58302266699273</v>
+        <v>41.58302287028404</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>1.91652321707221</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.366566479670305</v>
+        <v>0.3665664793619356</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>49.24034782780798</v>
+        <v>49.24034786951353</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>30.8530374509283</v>
+        <v>30.85303742775909</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.37520077790923</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-0.2342485493946358</v>
+        <v>-0.2342485494787403</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>51.82695093379393</v>
+        <v>51.82695107909499</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>32.31130618802195</v>
+        <v>32.31130618606655</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.3125278343269877</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>-0.04948983584043432</v>
+        <v>-0.0494898359946207</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>522.7541565804908</v>
+        <v>522.7541565804914</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>54.5</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>50.90640579040686</v>
+        <v>50.9064065671094</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>17.21828633704896</v>
+        <v>17.21828635893301</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>3.192497051227178</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.1850356913765788</v>
+        <v>-0.1850356936192969</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>511.4733896006021</v>
+        <v>511.4733896006022</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>48.05</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>57.85587131126581</v>
+        <v>57.85587125886764</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>19.51798095088931</v>
+        <v>19.51798124017185</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.7283386577451325</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.08787671919133233</v>
+        <v>0.08787671941560327</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>54.05049187495794</v>
+        <v>54.05049239360016</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>12.59871554434059</v>
+        <v>12.59871574859665</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>1.27197822733779</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.1122603671155191</v>
+        <v>0.112260366635063</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>53.97361633735492</v>
+        <v>53.97361636044461</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>15.22478447187373</v>
+        <v>15.22478452783945</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.760617295114085</v>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>498.9441155752468</v>
+        <v>498.9441155752469</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>57.1</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>53.45838567121151</v>
+        <v>53.45838578341923</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>27.10638527073353</v>
+        <v>27.10638529283992</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.620056674341036</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.4813043390264591</v>
+        <v>0.4813043385218445</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>47.603247879543</v>
+        <v>47.60324791425037</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>29.26039307133874</v>
+        <v>29.26039312001981</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.8433100139456761</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-0.4819141839848768</v>
+        <v>-0.4819141840269294</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>488.8979104889937</v>
+        <v>488.8979104889923</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>39.9</v>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>50.50178363646307</v>
+        <v>50.50178383849371</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>12.71692597047239</v>
+        <v>12.71692599310894</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>1.074079888439611</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.05924687023204278</v>
+        <v>0.05924686989563591</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>39.37036986652829</v>
+        <v>39.37036976950325</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>21.50163664777957</v>
+        <v>21.50163673389562</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>1.345283816282502</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-9.32665288310271</v>
+        <v>-9.326652877636132</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>42.11470551030486</v>
+        <v>42.11470553976781</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>14.11400893755898</v>
+        <v>14.11400882668858</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.3423318568761622</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.04750364199866763</v>
+        <v>0.04750364185850131</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>475.3320772960382</v>
+        <v>475.3320772960381</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>61.8</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>44.35447911731011</v>
+        <v>44.35447932441674</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>13.00820832998108</v>
+        <v>13.0082083440585</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.7345672408259335</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.1066589062108509</v>
+        <v>0.1066589052016255</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2181,7 +2181,7 @@
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>474.8731161740701</v>
+        <v>474.87311617407</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>24.35</v>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>47.1197676563804</v>
+        <v>47.11976764704006</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>26.81735316039164</v>
+        <v>26.81735311674169</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.7158299275388671</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.07436470178972998</v>
+        <v>0.07436470181776422</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>474.7817464997959</v>
+        <v>474.7817464997961</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>6.07</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>57.655495290173</v>
+        <v>57.65549522409462</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>15.58556537373398</v>
+        <v>15.58556542444842</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.9334858343414639</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.03441299821458883</v>
+        <v>0.03441299823140815</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>52.26987111771572</v>
+        <v>52.26987113908917</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>29.94338307506749</v>
+        <v>29.9433830812542</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.3688200112431441</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>-0.01366763528286369</v>
+        <v>-0.01366763529127343</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>459.4098730152714</v>
+        <v>459.409873015272</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>1880</v>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>40.06283616390967</v>
+        <v>40.06283617152327</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>16.71172429484598</v>
+        <v>16.71172430776101</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.6229934965662307</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-19.20419345481692</v>
+        <v>-19.20419345565777</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>442.4270914848673</v>
+        <v>442.4270914848674</v>
       </c>
       <c r="E37" s="2" t="n">
         <v>105</v>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>41.8448105376739</v>
+        <v>41.84481047671661</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>24.88002216419947</v>
+        <v>24.88002206677067</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.8087478741629615</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-1.871138257277019</v>
+        <v>-1.871138256988744</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>46.11781235547103</v>
+        <v>46.11781232923101</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>15.806142562236</v>
+        <v>15.80614252850291</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.256082269905151</v>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>47.23610138580127</v>
+        <v>47.23610138779281</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>28.78978311085551</v>
+        <v>28.78978323114167</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.1746813324909014</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-1.552702538676902</v>
+        <v>-1.552702538704937</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2569,7 +2569,7 @@
         <v>45.24331630944906</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>18.08951226580136</v>
+        <v>18.08951223306016</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>1.04372566316102</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-0.8614604637152564</v>
+        <v>-0.8614604634349099</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2605,7 +2605,7 @@
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>419.5353059649169</v>
+        <v>419.535305964917</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>9.98</v>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>42.04131901071852</v>
+        <v>42.04131912981686</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>26.72678014602368</v>
+        <v>26.72678014114166</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.335975109515038</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.008366818773398399</v>
+        <v>-0.008366818801431364</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>54.69770648794883</v>
+        <v>54.69770655720398</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>15.43045636843283</v>
+        <v>15.43045652107851</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>1.023829733570677</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.02129136438783163</v>
+        <v>0.02129136417162836</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>44.01760703854805</v>
+        <v>44.01760706696002</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>21.33494798698741</v>
+        <v>21.334948048315</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>1.031595582424542</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-2.410040754155257</v>
+        <v>-2.410040754435649</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>18.14864275051552</v>
+        <v>18.1486427607859</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>64.47578399552995</v>
+        <v>64.4757841204795</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.3745321416476234</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.2834025114022882</v>
+        <v>0.283402511178017</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>50.14212327714911</v>
+        <v>50.14212334628323</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>27.20710785675488</v>
+        <v>27.20710788008099</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.8661811693613135</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.05163714102956696</v>
+        <v>-0.05163714108563405</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>46.24856619186897</v>
+        <v>46.24856640513075</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>30.09459504828553</v>
+        <v>30.09459504828554</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.5985639926676436</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-0.008811208073448538</v>
+        <v>-0.008811208171568833</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>38.27425107882759</v>
+        <v>38.27425112831997</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>27.1713216926055</v>
+        <v>27.17132169172377</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>1.248760791605791</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>44.1681594067116</v>
+        <v>44.16815940330535</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>30.88617360007971</v>
+        <v>30.88617366113</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.2927270027077626</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.9076564463268855</v>
+        <v>-0.9076564463408987</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>43.10934075832134</v>
+        <v>43.10934133837628</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>28.86344158095253</v>
+        <v>28.86344156419235</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.4570071315006982</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.08714042178454223</v>
+        <v>0.08714042181257498</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>43.94967721138834</v>
+        <v>43.94967718639074</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>11.16674482071125</v>
+        <v>11.16674480571933</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.7724666649442282</v>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>47.77985935728047</v>
+        <v>47.77985919202784</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>13.84089946326911</v>
+        <v>13.84089953364152</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>1.853771204673815</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.4064827929479835</v>
+        <v>-0.4064827904249346</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>369.6497012691836</v>
+        <v>369.6497012691824</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>44.4</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>50.18577418024257</v>
+        <v>50.18577418287184</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>7.474352903642559</v>
+        <v>7.474353013268444</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.6480589829337459</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.003918341158777761</v>
+        <v>-0.003918341292237004</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>45.80555365200031</v>
+        <v>45.80555380631448</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>24.3296476542161</v>
+        <v>24.32964771238132</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.5301168375327538</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-1.470456768744411</v>
+        <v>-1.470456769865764</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>355.863404963521</v>
+        <v>355.8634049635206</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>28.2</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>44.90268730373873</v>
+        <v>44.90268883951885</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>19.14537746212603</v>
+        <v>19.14537779655351</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>1.870816255095116</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.06862061532379116</v>
+        <v>0.06862061338801345</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>349.4688240525206</v>
+        <v>349.4688240525208</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>81.3</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>33.6350617425975</v>
+        <v>33.63506180815695</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>31.4733995995488</v>
+        <v>31.47339974828258</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.7577526632333104</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.2866701126083626</v>
+        <v>0.2866701120336694</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>44.02262255554795</v>
+        <v>44.02262256940617</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>16.37298281884591</v>
+        <v>16.37298297598572</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>1.551163132568259</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-2.46102962674316</v>
+        <v>-2.461029626939404</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>347.6933913036669</v>
+        <v>347.6933913036668</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>29.4</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>38.50390316732724</v>
+        <v>38.50390292927064</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>13.67564526262068</v>
+        <v>13.67564552417415</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.7801535217607619</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.1381623606411645</v>
+        <v>-0.1381623604449276</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>344.5105095668258</v>
+        <v>344.5105095668257</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>67.7</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>46.3285059041681</v>
+        <v>46.32850585913553</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>23.32840468587395</v>
+        <v>23.32840446891599</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.2193044977159437</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.1042137844074038</v>
+        <v>0.104213783986894</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>338.4180120933575</v>
+        <v>338.4180120933576</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>177</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>26.54916422087081</v>
+        <v>26.5491642821348</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>26.48924177055491</v>
+        <v>26.48924174360583</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.750165316765388</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-1.352097255742629</v>
+        <v>-1.352097255854746</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>41.32348398716119</v>
+        <v>41.32348400249761</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>19.18635307887863</v>
+        <v>19.18635335952536</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.4009966140390467</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.5662028650649406</v>
+        <v>-0.5662028650929661</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>330.8222654617473</v>
+        <v>330.8222654617468</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>19.45</v>
@@ -3679,7 +3679,7 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>47.46911794695054</v>
+        <v>47.46911821193017</v>
       </c>
       <c r="I61" s="2" t="n">
         <v>13.28982047966328</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.02403068622756863</v>
+        <v>-0.02403068646586065</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>46.82090170459927</v>
+        <v>46.82090169690601</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>18.41214582093743</v>
+        <v>18.41214579099832</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.2286572105170016</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.5644588582103581</v>
+        <v>-0.5644588581402706</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3771,7 +3771,7 @@
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>325.2703774014073</v>
+        <v>325.2703774014061</v>
       </c>
       <c r="E63" s="2" t="n">
         <v>74.3</v>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>36.60218295098283</v>
+        <v>36.60218300323436</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>17.65194106342507</v>
+        <v>17.65194107749953</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.3678364364167878</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.814952893531141</v>
+        <v>-0.8149528931106431</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>45.93876062673137</v>
+        <v>45.93876067276577</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>30.42464118011972</v>
+        <v>30.42464118025633</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.9079523187005889</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-12.29579161094156</v>
+        <v>-12.29579161178254</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>39.28043427404442</v>
+        <v>39.28043422066354</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>21.25291059009146</v>
+        <v>21.2529106676058</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.2102217793858742</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-1.724492716345079</v>
+        <v>-1.724492715868487</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>50.13758956766841</v>
+        <v>50.13758914980431</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>24.78789276130733</v>
+        <v>24.78789291963687</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.5386565802160797</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.214746841168152</v>
+        <v>-0.2147468407837888</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>51.63431288306025</v>
+        <v>51.63431289717074</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>32.20069310143391</v>
+        <v>32.20069316004242</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4025606890735801</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.1738023744839139</v>
+        <v>0.1738023745119473</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>42.05539251160287</v>
+        <v>42.05539260995853</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>17.07120798668088</v>
+        <v>17.07120829019643</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.904018293317979</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.2234359651077971</v>
+        <v>-0.2234359654722362</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>37.02351429036546</v>
+        <v>37.02351431543109</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>39.95172840417597</v>
+        <v>39.95172834377799</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.3736175337522871</v>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>49.27933149612411</v>
+        <v>49.27933195536085</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>26.54081336346389</v>
+        <v>26.54081330868603</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.3021083385677799</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.01279963991715352</v>
+        <v>0.01279963983304803</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>37.73710052447799</v>
+        <v>37.73710188407084</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>7.578239942429825</v>
+        <v>7.578240085761617</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.6903404347948481</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.03234129013699305</v>
+        <v>0.03234128971648209</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>302.2398939513393</v>
+        <v>302.2398939512961</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>41.3</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>39.50043926202966</v>
+        <v>39.50043939230526</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>12.36700622319114</v>
+        <v>12.36700616011662</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.7583543671928425</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.1377093085410869</v>
+        <v>-0.1377093086672437</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4301,7 +4301,7 @@
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>302.0798237348229</v>
+        <v>302.0798237348239</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>19.75</v>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>40.00589299954748</v>
+        <v>40.00589313398149</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>20.0719619942676</v>
+        <v>20.07196208662345</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.8314611749119293</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.04729823666129725</v>
+        <v>-0.04729823671736576</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>298.2875750965616</v>
+        <v>298.2875750965622</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>8.65</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>48.02539058810623</v>
+        <v>48.02539065624134</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>31.60943063434203</v>
+        <v>31.60943069027834</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.6095204455587635</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.003609390500986409</v>
+        <v>-0.003609390523413455</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>26.86804444221994</v>
+        <v>26.86804446679413</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>26.31862807322475</v>
+        <v>26.3186281424945</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>1.065416436243068</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-4.333035127112247</v>
+        <v>-4.333035129354993</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>40.93627450698609</v>
+        <v>40.93627449022115</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>23.72262429826972</v>
+        <v>23.72262434398222</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.8683105312073887</v>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>24.76832138047335</v>
+        <v>24.76832143456805</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>50.17979962236757</v>
+        <v>50.17979950574679</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.1761600127597839</v>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>289.3931012764559</v>
+        <v>289.3931012764545</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>20.15</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>35.41486829247042</v>
+        <v>35.41486839764082</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>16.99907819781869</v>
+        <v>16.99907830440848</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.8229910077504513</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.0760333632884852</v>
+        <v>-0.07603336340062117</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,7 +4633,7 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>50.49351134911474</v>
+        <v>50.49351133402477</v>
       </c>
       <c r="I79" s="2" t="n">
         <v>5.73845682913478</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-1.945536004825834</v>
+        <v>-1.945536003760545</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>276.7946915117267</v>
+        <v>276.794691511727</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>46.7</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>42.85380403458104</v>
+        <v>42.85380407989482</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>10.10055283827799</v>
+        <v>10.10055281175142</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>3.163889474794347</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.3346762827984709</v>
+        <v>-0.3346762831068408</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>28.12497177823154</v>
+        <v>28.12497173918491</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>43.98126014125751</v>
+        <v>43.98126012165837</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.1260589222536288</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.05023570405381628</v>
+        <v>0.0502357041939866</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,7 +4792,7 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>35.81367276691375</v>
+        <v>35.8136727780937</v>
       </c>
       <c r="I82" s="2" t="n">
         <v>26.97669105808152</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-1.479100798129205</v>
+        <v>-1.479100798143226</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>33.91437623029201</v>
+        <v>33.91437633709279</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>20.53228615543403</v>
+        <v>20.5322861792567</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.4057153361421413</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-3.347800660431654</v>
+        <v>-3.347800660291504</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>264.001670648683</v>
+        <v>264.0016706486824</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>20.35</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>33.98528326136606</v>
+        <v>33.98528309441124</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>35.96020156185598</v>
+        <v>35.96020154106276</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>1.244751897517626</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.03543465313260941</v>
+        <v>-0.03543465300645482</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>51.65384851343826</v>
+        <v>51.65384851620011</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>21.25793869606789</v>
+        <v>21.25793879491265</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.1145242560780299</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.2192719957535324</v>
+        <v>-0.2192719958376314</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>258.1205648875545</v>
+        <v>258.1205648875547</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>32.55</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>43.83377461967024</v>
+        <v>43.83377453845731</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>24.17382213224707</v>
+        <v>24.1738222779786</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.4968641409156804</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.3165838958085204</v>
+        <v>-0.316583894350752</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>54.800279927151</v>
+        <v>54.80028029691951</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>18.28257218757575</v>
+        <v>18.28257214900536</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.963719827376367</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.7843235394209975</v>
+        <v>0.7843235374586224</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>255.8281121450803</v>
+        <v>255.8281121450804</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>2.9</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>50.38294863352041</v>
+        <v>50.38294863559409</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>4.623676406529136</v>
+        <v>4.623676404559654</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.5815954787037995</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.04190171941732529</v>
+        <v>-0.04190171942012888</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>253.5602076817368</v>
+        <v>253.5602076817361</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>125</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>39.31770868245531</v>
+        <v>39.31770887614021</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>23.06136436378518</v>
+        <v>23.0613644482053</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.3738271444984303</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-2.181594199691157</v>
+        <v>-2.181594200251832</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>244.7463062375292</v>
+        <v>244.7463062375299</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>44.5</v>
@@ -5219,7 +5219,7 @@
         <v>42.36321756909849</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>18.75067654923309</v>
+        <v>18.75067660469487</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.3253733246469661</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.5757832509943052</v>
+        <v>-0.5757832510363554</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>41.31554964942543</v>
+        <v>41.3155497037858</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>12.84795213917887</v>
+        <v>12.84795216546368</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.4923774439834016</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.3053859219986216</v>
+        <v>-0.3053859219565708</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>239.137383720026</v>
+        <v>239.1373837200259</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>291.5</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>37.84693190428838</v>
+        <v>37.84693192069421</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>15.65089672684538</v>
+        <v>15.65089677119456</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.748161642941366</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-2.677513722988849</v>
+        <v>-2.677513723829905</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5350,21 +5350,21 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>8488</v>
+        <v>8466</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>吉源-KY</t>
+          <t>美吉吉-KY</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>239.0701513992827</v>
+        <v>238.593012589109</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>9.24</v>
+        <v>14.9</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>49.52163055940701</v>
+        <v>45.43712552020452</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>22.51632876046137</v>
+        <v>15.98701964027589</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>1.281590585841818</v>
+        <v>0.5657884665941212</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.1055033996341257</v>
+        <v>-0.01510060466278614</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, adx_trending</t>
+          <t>avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>8466</v>
+        <v>8087</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>美吉吉-KY</t>
+          <t>華鎂鑫</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>238.593012589109</v>
+        <v>237.5603722103005</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>14.9</v>
+        <v>22.4</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>45.4371256562962</v>
+        <v>47.03531361922868</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>15.98701958534786</v>
+        <v>3.870230853810646</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.5657884665941212</v>
+        <v>0.06548518569400559</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.01510060476090434</v>
+        <v>-0.0494459207886373</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>8087</v>
+        <v>9136</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>華鎂鑫</t>
+          <t>巨騰-DR</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>237.5603722103005</v>
+        <v>237.367569388544</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>22.4</v>
+        <v>7.68</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,16 +5481,16 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>47.03531368844032</v>
+        <v>15.69743694805263</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>3.870230723404996</v>
+        <v>21.72441349219234</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.06548518569400559</v>
+        <v>3.421454116568932</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.0494459210409437</v>
+        <v>-0.0615230871017084</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>9136</v>
+        <v>8049</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>巨騰-DR</t>
+          <t>晶采</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>237.3675693885414</v>
+        <v>233.035754866115</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>7.68</v>
+        <v>23.9</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>15.69743698809964</v>
+        <v>33.36078612502395</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>21.72441319197193</v>
+        <v>16.52441077231297</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>3.421454116568932</v>
+        <v>1.109337734460097</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.06152308711852905</v>
+        <v>-0.04219644784128115</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>volume_break, avoid_chase, adx_trending</t>
+          <t>avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>8049</v>
+        <v>8374</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>晶采</t>
+          <t>羅昇</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>233.0357548661148</v>
+        <v>227.2064023171831</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>23.9</v>
+        <v>70.5</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>33.36078602466803</v>
+        <v>32.59237334967027</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>16.52441081117911</v>
+        <v>18.33774773471264</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>1.109337734460097</v>
+        <v>1.483481291786557</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.04219644779923101</v>
+        <v>-0.2881683011987934</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5615,21 +5615,21 @@
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>8374</v>
+        <v>8091</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>羅昇</t>
+          <t>翔名</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>227.2064023171833</v>
+        <v>226.60458783002</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>70.5</v>
+        <v>200</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>32.59237327679445</v>
+        <v>34.83051942503594</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>18.33774776030779</v>
+        <v>14.6596533864364</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>1.483481291786557</v>
+        <v>1.350645171258896</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.2881683004979345</v>
+        <v>-2.401277663960208</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, stronger_than_market</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>8091</v>
+        <v>8131</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>翔名</t>
+          <t>福懋科</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>226.60458783002</v>
+        <v>224.2324896292183</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>200</v>
+        <v>60.7</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>34.83051939179053</v>
+        <v>42.81572559547568</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>14.659653357029</v>
+        <v>15.94898322427475</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>1.350645171258896</v>
+        <v>0.5436698798860434</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-2.401277663960208</v>
+        <v>-0.4495956371014578</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok</t>
+          <t>avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>8131</v>
+        <v>8455</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>福懋科</t>
+          <t>大拓-KY</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>224.2324896291973</v>
+        <v>221.4752405649225</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>60.7</v>
+        <v>0</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>42.81572559001732</v>
+        <v>41.54577427135298</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>15.94898320783668</v>
+        <v>9.381552309195829</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.5436698798860434</v>
+        <v>0</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.4495956370874426</v>
+        <v>-0.5790421247135346</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>8455</v>
+        <v>8121</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>大拓-KY</t>
+          <t>越峰</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>221.4752405649225</v>
+        <v>220.0969304012783</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>0</v>
+        <v>28.8</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>41.54577426277354</v>
+        <v>42.33815247367959</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>9.381552307582728</v>
+        <v>24.36864468633437</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0</v>
+        <v>0.4307129207862044</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.5790421242790109</v>
+        <v>-0.4964161952795031</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>obv_uptrend, mfi_strong</t>
+          <t>avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>8121</v>
+        <v>8043</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>越峰</t>
+          <t>蜜望實</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>220.0969304012787</v>
+        <v>216.7625187200225</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>28.8</v>
+        <v>132</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>42.33815217051502</v>
+        <v>44.42479915145969</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>24.36864468633437</v>
+        <v>16.68096056319099</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.4307129207862044</v>
+        <v>0.697833294412044</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.4964161948730111</v>
+        <v>-0.7924920195058782</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>8043</v>
+        <v>8478</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>蜜望實</t>
+          <t>東哥遊艇</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>216.7625187200225</v>
+        <v>215.7705829046616</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>132</v>
+        <v>128.5</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,16 +5905,16 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>44.42479914754244</v>
+        <v>19.73839964408349</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>16.68096046317009</v>
+        <v>21.05455580993478</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.697833294412044</v>
+        <v>2.977058290466164</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.7924920194498373</v>
+        <v>-0.8966102709533466</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok</t>
+          <t>volume_break, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>8478</v>
+        <v>8114</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>東哥遊艇</t>
+          <t>振樺電</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>215.7705829046616</v>
+        <v>213.1119035547726</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>128.5</v>
+        <v>178</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,16 +5958,16 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>19.73839977360663</v>
+        <v>44.55643560850005</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>21.05455586292065</v>
+        <v>15.08285076300987</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>2.977058290466164</v>
+        <v>1.070775557214398</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.8966102716541926</v>
+        <v>0.6491751544239834</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>volume_break, avoid_chase, adx_trending</t>
+          <t>avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>8114</v>
+        <v>8481</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>振樺電</t>
+          <t>政伸</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>213.1119035547726</v>
+        <v>212.6587828790156</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>178</v>
+        <v>40.05</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,16 +6011,16 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>44.55643529092183</v>
+        <v>39.52979480258529</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>15.08285084591003</v>
+        <v>16.0616949236978</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>1.070775557214398</v>
+        <v>0.8395852968897267</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L105" s="2" t="n">
         <v>0</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.6491751576478841</v>
+        <v>-0.05714974789666832</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6039,21 +6039,21 @@
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>8481</v>
+        <v>8291</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>政伸</t>
+          <t>尚茂</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>212.6587828790156</v>
+        <v>201.8857501771712</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>40.05</v>
+        <v>23.2</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>39.52979441482393</v>
+        <v>38.68801316322939</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>16.0616949236978</v>
+        <v>18.79162327717224</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.8395852968897267</v>
+        <v>0.3369283660276646</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.05714974789666832</v>
+        <v>-0.3482249730297058</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6092,21 +6092,21 @@
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>8291</v>
+        <v>8176</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>尚茂</t>
+          <t>智捷</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>201.8857501771712</v>
+        <v>196.9963980211896</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>23.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>38.68801316322939</v>
+        <v>45.36114131898143</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>18.79162327717224</v>
+        <v>17.69447054557772</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.3369283660276646</v>
+        <v>0.2062662338911171</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.3482249730297058</v>
+        <v>0.01126038990997359</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6145,21 +6145,21 @@
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>8176</v>
+        <v>9955</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>智捷</t>
+          <t>佳龍</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>196.9963980211895</v>
+        <v>184.4653787851462</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>9.699999999999999</v>
+        <v>21.75</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,16 +6170,16 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>45.36114131898143</v>
+        <v>30.08629102429592</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>17.69447047091241</v>
+        <v>16.25319483740504</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.2062662338911171</v>
+        <v>4.34653787851462</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.01126038992399189</v>
+        <v>-0.1439504952306802</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, stronger_than_market</t>
+          <t>volume_break, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>9955</v>
+        <v>8488</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>佳龍</t>
+          <t>吉源-KY</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>184.4653787851462</v>
+        <v>179.0701513992827</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>21.75</v>
+        <v>9.24</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,16 +6223,16 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>30.08629146061122</v>
+        <v>49.52162960943582</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>16.2531948047989</v>
+        <v>22.51632558766489</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>4.34653787851462</v>
+        <v>1.281590585841818</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L109" s="2" t="n">
         <v>0</v>
@@ -6241,11 +6241,11 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.1439504955530714</v>
+        <v>0.105503402886064</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>volume_break, avoid_chase</t>
+          <t>avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>39.35144233586585</v>
+        <v>39.35144245057565</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>12.43360502172857</v>
+        <v>12.43360509723093</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.8463595253290574</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.06077418353378095</v>
+        <v>-0.06077418355602493</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,7 +6329,7 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>40.81778808623167</v>
+        <v>40.81778814137117</v>
       </c>
       <c r="I111" s="2" t="n">
         <v>18.26757285832872</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.1120079416400159</v>
+        <v>-0.1120079417942023</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>159.3744542584215</v>
+        <v>159.3744542584212</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>25.7</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>34.34670886196825</v>
+        <v>34.34670880173452</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>24.01437842929512</v>
+        <v>24.01437846864729</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.7812393633364673</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.1677220524579703</v>
+        <v>-0.1677220525140365</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>34.3887451989589</v>
+        <v>34.38874522397954</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>20.25953174821339</v>
+        <v>20.25953178449305</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>1.432971404249287</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.1165597919716665</v>
+        <v>-0.116559791957649</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>45.72098936937811</v>
+        <v>45.72098935078875</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>10.98233258518944</v>
+        <v>10.98233257494084</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.6110869998767769</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.08801990038189146</v>
+        <v>-0.08801990036787458</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>153.2380025856971</v>
+        <v>153.2380025856979</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>225.5</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>42.63571438201638</v>
+        <v>42.63571452536123</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>6.805051810590511</v>
+        <v>6.805051835038824</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>1.532711222355678</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-2.385427868927003</v>
+        <v>-2.385427872851752</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6580,7 +6580,7 @@
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>152.18462500078</v>
+        <v>152.1846250007802</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>89.2</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>43.46139615292083</v>
+        <v>43.46139766520327</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>13.32812679622607</v>
+        <v>13.3281270178001</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.7739671052068966</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.03284155341458872</v>
+        <v>-0.03284155869956074</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>118.0659889900677</v>
+        <v>118.0659889900678</v>
       </c>
       <c r="E117" s="2" t="n">
         <v>87.5</v>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>35.50775766789729</v>
+        <v>35.50775770441446</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>16.90053599948205</v>
+        <v>16.90053602115409</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>1.101770488523073</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.08898545778684763</v>
+        <v>-0.08898545798307289</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>115.3784983961149</v>
+        <v>115.3784983961148</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>66.7</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>23.66743973869228</v>
+        <v>23.66743969201558</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>16.3325111402477</v>
+        <v>16.33251109738916</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>1.017304367681117</v>
@@ -6753,7 +6753,7 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>37.08367391625161</v>
+        <v>37.08367412357857</v>
       </c>
       <c r="I119" s="2" t="n">
         <v>11.53810276170083</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.01753516390825852</v>
+        <v>-0.01753516397834326</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>104.3631957117807</v>
+        <v>104.3631957117804</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>37.6</v>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>33.84733019979352</v>
+        <v>33.84733019421348</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>19.31726155362415</v>
+        <v>19.31726162669893</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>1.663421211349669</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.02069686114624836</v>
+        <v>-0.02069686135650006</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>

</xml_diff>